<commit_message>
First stages of fixing extraction pipeline.
</commit_message>
<xml_diff>
--- a/thesis/Word Count Tracker.xlsx
+++ b/thesis/Word Count Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\wesle\biomedical_kg_thesis\thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719647DD-2FB2-4A66-B5F7-EB2947207B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDDAC44D-483B-4CFB-BF8D-B3683335F09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1875" windowWidth="29040" windowHeight="15840" xr2:uid="{9A934C0C-D068-49A2-992C-A9C72EA321F1}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
     <t>Count</t>
   </si>
@@ -100,6 +100,30 @@
   </si>
   <si>
     <t>Daily Target</t>
+  </si>
+  <si>
+    <t>Abstract</t>
+  </si>
+  <si>
+    <t>Introduction</t>
+  </si>
+  <si>
+    <t>Lit. Review</t>
+  </si>
+  <si>
+    <t>Methodology</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>Discussion</t>
+  </si>
+  <si>
+    <t>Conclusion</t>
+  </si>
+  <si>
+    <t>Section Counts</t>
   </si>
 </sst>
 </file>
@@ -199,7 +223,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -387,11 +411,132 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -455,6 +600,22 @@
     <xf numFmtId="3" fontId="1" fillId="10" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -463,8 +624,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFE1DECD"/>
       <color rgb="FFF49E9E"/>
-      <color rgb="FFE1DECD"/>
       <color rgb="FFFFFF99"/>
       <color rgb="FF63BE7B"/>
       <color rgb="FFFFEB84"/>
@@ -711,7 +872,7 @@
                   <c:v>5610</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5786</c:v>
+                  <c:v>5988</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1576,7 +1737,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>219808</xdr:colOff>
+      <xdr:colOff>419100</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1923,7 +2084,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EA3A3B3-C19C-41F0-9C7A-3F939AAD4664}">
-  <dimension ref="B1:K27"/>
+  <dimension ref="B1:P27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.85546875" style="24" customWidth="1"/>
@@ -1937,10 +2098,15 @@
     <col min="9" max="9" width="2.85546875" style="24" customWidth="1"/>
     <col min="10" max="10" width="27.140625" style="24" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.85546875" style="24" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="24"/>
+    <col min="12" max="12" width="3.5703125" style="24" customWidth="1"/>
+    <col min="13" max="13" width="12.85546875" style="24" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" style="24"/>
+    <col min="15" max="15" width="11.42578125" style="24" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.42578125" style="24" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
       <c r="D1" s="24"/>
@@ -1948,7 +2114,7 @@
       <c r="F1" s="24"/>
       <c r="G1" s="24"/>
     </row>
-    <row r="2" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="32" t="s">
         <v>1</v>
       </c>
@@ -1977,8 +2143,14 @@
         <f>COUNTIF(C3:C27, "")</f>
         <v>18</v>
       </c>
+      <c r="M2" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" s="51"/>
+      <c r="O2" s="51"/>
+      <c r="P2" s="52"/>
     </row>
-    <row r="3" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="3">
         <v>46250</v>
       </c>
@@ -2007,8 +2179,20 @@
         <f>COUNTIF(C3:C19, "")</f>
         <v>10</v>
       </c>
+      <c r="M3" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="N3" s="43">
+        <v>0</v>
+      </c>
+      <c r="O3" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="43">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
         <v>46251</v>
       </c>
@@ -2038,10 +2222,22 @@
       </c>
       <c r="K4" s="12" cm="1">
         <f t="array" ref="K4">MAX(0,20000-LOOKUP(2,1/(C3:C27&lt;&gt;""),C3:C27))</f>
-        <v>14214</v>
+        <v>14012</v>
+      </c>
+      <c r="M4" s="48" t="s">
+        <v>14</v>
+      </c>
+      <c r="N4" s="44">
+        <v>0</v>
+      </c>
+      <c r="O4" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="P4" s="44">
+        <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2">
         <v>46252</v>
       </c>
@@ -2071,10 +2267,22 @@
       </c>
       <c r="K5" s="9">
         <f>ROUNDUP(K4/K3,0)</f>
-        <v>1422</v>
+        <v>1402</v>
+      </c>
+      <c r="M5" s="48" t="s">
+        <v>15</v>
+      </c>
+      <c r="N5" s="44">
+        <v>5610</v>
+      </c>
+      <c r="O5" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="P5" s="45">
+        <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2">
         <v>46253</v>
       </c>
@@ -2104,10 +2312,18 @@
       </c>
       <c r="K6" s="8">
         <f>ROUNDUP(K4/K2,0)</f>
-        <v>790</v>
-      </c>
+        <v>779</v>
+      </c>
+      <c r="M6" s="49" t="s">
+        <v>16</v>
+      </c>
+      <c r="N6" s="45">
+        <v>378</v>
+      </c>
+      <c r="O6" s="46"/>
+      <c r="P6" s="46"/>
     </row>
-    <row r="7" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B7" s="4">
         <v>46254</v>
       </c>
@@ -2133,7 +2349,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B8" s="2">
         <v>46255</v>
       </c>
@@ -2159,24 +2375,25 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="9" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="2">
         <v>46256</v>
       </c>
       <c r="C9" s="40">
-        <v>5786</v>
+        <f>SUM(P3:P5,N3:N6)</f>
+        <v>5988</v>
       </c>
       <c r="D9" s="26">
         <f t="shared" si="1"/>
-        <v>176</v>
+        <v>378</v>
       </c>
       <c r="E9" s="26">
         <f t="shared" si="2"/>
-        <v>1214</v>
+        <v>1012</v>
       </c>
       <c r="F9" s="27">
         <f t="shared" ref="F9:F27" si="3">IF(G9="","",IF(C9="","",D9/(G9-C8)))</f>
-        <v>0.12661870503597122</v>
+        <v>0.27194244604316548</v>
       </c>
       <c r="G9" s="35">
         <v>7000</v>
@@ -2185,7 +2402,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="10" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B10" s="4">
         <v>46257</v>
       </c>
@@ -2207,7 +2424,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B11" s="2">
         <v>46258</v>
       </c>
@@ -2229,7 +2446,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B12" s="2">
         <v>46259</v>
       </c>
@@ -2251,7 +2468,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B13" s="2">
         <v>46260</v>
       </c>
@@ -2273,7 +2490,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="14" spans="2:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:16" ht="15" x14ac:dyDescent="0.25">
       <c r="B14" s="4">
         <v>46261</v>
       </c>
@@ -2295,7 +2512,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B15" s="2">
         <v>46262</v>
       </c>
@@ -2317,7 +2534,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B16" s="2">
         <v>46263</v>
       </c>
@@ -2582,7 +2799,9 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <mergeCells count="1">
+    <mergeCell ref="M2:P2"/>
+  </mergeCells>
   <conditionalFormatting sqref="D4:D27">
     <cfRule type="colorScale" priority="3">
       <colorScale>

</xml_diff>

<commit_message>
Report & EPI progress.
</commit_message>
<xml_diff>
--- a/thesis/Word Count Tracker.xlsx
+++ b/thesis/Word Count Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\wesle\biomedical_kg_thesis\thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A66491DE-42E9-4CC2-B0F3-3B9BEF1318EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA35CD16-F248-4098-A12C-C3ABF73C2BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1875" windowWidth="29040" windowHeight="15840" xr2:uid="{9A934C0C-D068-49A2-992C-A9C72EA321F1}"/>
   </bookViews>
@@ -36,28 +36,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -950,7 +928,10 @@
                   <c:v>7218</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>7753</c:v>
+                  <c:v>8459</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8459</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2219,7 +2200,7 @@
       </c>
       <c r="K2" s="10">
         <f>COUNTIF(C3:C27, "")</f>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M2" s="58" t="s">
         <v>20</v>
@@ -2255,7 +2236,7 @@
       </c>
       <c r="K3" s="11">
         <f>COUNTIF(C3:C19, "")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M3" s="46" t="s">
         <v>13</v>
@@ -2298,9 +2279,9 @@
       <c r="J4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="K4" s="12" cm="1">
-        <f t="array" ref="K4">MAX(0,20000-LOOKUP(2,1/(C3:C27&lt;&gt;""),C3:C27))</f>
-        <v>12247</v>
+      <c r="K4" s="12">
+        <f>MAX(0,20000-P6)</f>
+        <v>11541</v>
       </c>
       <c r="M4" s="47" t="s">
         <v>14</v>
@@ -2345,13 +2326,13 @@
       </c>
       <c r="K5" s="9">
         <f>ROUNDUP(K4/K3,0)</f>
-        <v>1750</v>
+        <v>1924</v>
       </c>
       <c r="M5" s="47" t="s">
         <v>15</v>
       </c>
       <c r="N5" s="44">
-        <v>5612</v>
+        <v>5614</v>
       </c>
       <c r="O5" s="54" t="s">
         <v>19</v>
@@ -2390,20 +2371,20 @@
       </c>
       <c r="K6" s="8">
         <f>ROUNDUP(K4/K2,0)</f>
-        <v>817</v>
+        <v>825</v>
       </c>
       <c r="M6" s="48" t="s">
         <v>16</v>
       </c>
       <c r="N6" s="45">
-        <v>2141</v>
+        <v>2845</v>
       </c>
       <c r="O6" s="56" t="s">
         <v>21</v>
       </c>
       <c r="P6" s="57">
         <f>SUM($P$3:$P$5,$N$3:$N$6)</f>
-        <v>7753</v>
+        <v>8459</v>
       </c>
     </row>
     <row r="7" spans="2:16" ht="15" x14ac:dyDescent="0.25">
@@ -2541,20 +2522,19 @@
         <v>46259</v>
       </c>
       <c r="C12" s="41">
-        <f>P6</f>
-        <v>7753</v>
+        <v>8459</v>
       </c>
       <c r="D12" s="28">
         <f t="shared" si="1"/>
-        <v>535</v>
+        <v>1241</v>
       </c>
       <c r="E12" s="28">
         <f t="shared" si="2"/>
-        <v>747</v>
+        <v>41</v>
       </c>
       <c r="F12" s="33">
         <f t="shared" si="3"/>
-        <v>0.41731669266770671</v>
+        <v>0.96801872074883</v>
       </c>
       <c r="G12" s="36">
         <v>8500</v>
@@ -2567,20 +2547,25 @@
       <c r="B13" s="2">
         <v>46260</v>
       </c>
-      <c r="C13" s="40"/>
-      <c r="D13" s="26" t="str">
+      <c r="C13" s="40">
+        <f>P6</f>
+        <v>8459</v>
+      </c>
+      <c r="D13" s="26">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E13" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="E13" s="26">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F13" s="27" t="str">
+        <v>1541</v>
+      </c>
+      <c r="F13" s="27">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="G13" s="35"/>
+        <v>0</v>
+      </c>
+      <c r="G13" s="35">
+        <v>10000</v>
+      </c>
       <c r="H13" s="19">
         <v>20000</v>
       </c>

</xml_diff>

<commit_message>
Report progress & backup.
</commit_message>
<xml_diff>
--- a/thesis/Word Count Tracker.xlsx
+++ b/thesis/Word Count Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\wesle\biomedical_kg_thesis\thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7180AE4A-15A2-4C69-928C-D034CF6F94B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A573B77-8F23-4118-9FA3-4252068B2F4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="300" windowWidth="29040" windowHeight="15840" xr2:uid="{9A934C0C-D068-49A2-992C-A9C72EA321F1}"/>
   </bookViews>
@@ -664,6 +664,15 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -672,15 +681,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="1" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="1" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="2" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -954,6 +954,18 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>9647</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>9647</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>9647</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>9647</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>11228</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2227,14 +2239,14 @@
       </c>
       <c r="L2" s="10">
         <f>COUNTIF(C3:C27, "")</f>
-        <v>13</v>
-      </c>
-      <c r="N2" s="58" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="Q2" s="60"/>
+      <c r="O2" s="66"/>
+      <c r="P2" s="66"/>
+      <c r="Q2" s="67"/>
     </row>
     <row r="3" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="3">
@@ -2252,7 +2264,7 @@
       <c r="F3" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="61"/>
+      <c r="G3" s="58"/>
       <c r="H3" s="25" t="s">
         <v>8</v>
       </c>
@@ -2264,7 +2276,7 @@
       </c>
       <c r="L3" s="11">
         <f>COUNTIF(C3:C19, "")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N3" s="46" t="s">
         <v>13</v>
@@ -2291,15 +2303,15 @@
         <v>841</v>
       </c>
       <c r="E4" s="26">
-        <f>IF(C4="", "", H4-C4)</f>
+        <f t="shared" ref="E4:E27" si="0">IF(C4="", "", H4-C4)</f>
         <v>-165</v>
       </c>
       <c r="F4" s="27">
-        <f>IF(H4="","",IF(C4="","",D4/(H4-C3)))</f>
+        <f t="shared" ref="F4:F27" si="1">IF(H4="","",IF(C4="","",D4/(H4-C3)))</f>
         <v>1.2440828402366864</v>
       </c>
-      <c r="G4" s="63">
-        <f t="shared" ref="G4:G13" si="0">H4-C3</f>
+      <c r="G4" s="60">
+        <f t="shared" ref="G4:G13" si="2">H4-C3</f>
         <v>676</v>
       </c>
       <c r="H4" s="35">
@@ -2313,7 +2325,7 @@
       </c>
       <c r="L4" s="12">
         <f>MAX(0,20000-Q6)</f>
-        <v>10353</v>
+        <v>8772</v>
       </c>
       <c r="N4" s="47" t="s">
         <v>14</v>
@@ -2336,19 +2348,19 @@
         <v>2998</v>
       </c>
       <c r="D5" s="26">
-        <f t="shared" ref="D5:D27" si="1">IF(C5="", "", C5-C4)</f>
+        <f t="shared" ref="D5:D27" si="3">IF(C5="", "", C5-C4)</f>
         <v>633</v>
       </c>
       <c r="E5" s="26">
-        <f>IF(C5="", "", H5-C5)</f>
+        <f t="shared" si="0"/>
         <v>202</v>
       </c>
       <c r="F5" s="27">
-        <f>IF(H5="","",IF(C5="","",D5/(H5-C4)))</f>
+        <f t="shared" si="1"/>
         <v>0.75808383233532939</v>
       </c>
-      <c r="G5" s="63">
-        <f t="shared" si="0"/>
+      <c r="G5" s="60">
+        <f t="shared" si="2"/>
         <v>835</v>
       </c>
       <c r="H5" s="35">
@@ -2362,7 +2374,7 @@
       </c>
       <c r="L5" s="9">
         <f>ROUNDUP(L4/L3,0)</f>
-        <v>2071</v>
+        <v>8772</v>
       </c>
       <c r="N5" s="47" t="s">
         <v>15</v>
@@ -2385,19 +2397,19 @@
         <v>3611</v>
       </c>
       <c r="D6" s="26">
+        <f t="shared" si="3"/>
+        <v>613</v>
+      </c>
+      <c r="E6" s="26">
+        <f t="shared" si="0"/>
+        <v>389</v>
+      </c>
+      <c r="F6" s="27">
         <f t="shared" si="1"/>
-        <v>613</v>
-      </c>
-      <c r="E6" s="26">
-        <f>IF(C6="", "", H6-C6)</f>
-        <v>389</v>
-      </c>
-      <c r="F6" s="27">
-        <f>IF(H6="","",IF(C6="","",D6/(H6-C5)))</f>
         <v>0.61177644710578838</v>
       </c>
-      <c r="G6" s="63">
-        <f t="shared" si="0"/>
+      <c r="G6" s="60">
+        <f t="shared" si="2"/>
         <v>1002</v>
       </c>
       <c r="H6" s="35">
@@ -2411,20 +2423,20 @@
       </c>
       <c r="L6" s="8">
         <f>ROUNDUP(L4/L2,0)</f>
-        <v>797</v>
+        <v>975</v>
       </c>
       <c r="N6" s="48" t="s">
         <v>16</v>
       </c>
       <c r="O6" s="45">
-        <v>4025</v>
+        <v>5606</v>
       </c>
       <c r="P6" s="56" t="s">
         <v>21</v>
       </c>
       <c r="Q6" s="57">
         <f>SUM($Q$3:$Q$5,$O$3:$O$6)</f>
-        <v>9647</v>
+        <v>11228</v>
       </c>
     </row>
     <row r="7" spans="2:17" ht="15" x14ac:dyDescent="0.25">
@@ -2435,19 +2447,19 @@
         <v>5050</v>
       </c>
       <c r="D7" s="28">
+        <f t="shared" si="3"/>
+        <v>1439</v>
+      </c>
+      <c r="E7" s="28">
+        <f t="shared" si="0"/>
+        <v>-50</v>
+      </c>
+      <c r="F7" s="33">
         <f t="shared" si="1"/>
-        <v>1439</v>
-      </c>
-      <c r="E7" s="28">
-        <f>IF(C7="", "", H7-C7)</f>
-        <v>-50</v>
-      </c>
-      <c r="F7" s="33">
-        <f>IF(H7="","",IF(C7="","",D7/(H7-C6)))</f>
         <v>1.0359971202303815</v>
       </c>
-      <c r="G7" s="66">
-        <f t="shared" si="0"/>
+      <c r="G7" s="63">
+        <f t="shared" si="2"/>
         <v>1389</v>
       </c>
       <c r="H7" s="36">
@@ -2465,19 +2477,19 @@
         <v>5610</v>
       </c>
       <c r="D8" s="26">
+        <f t="shared" si="3"/>
+        <v>560</v>
+      </c>
+      <c r="E8" s="26">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="F8" s="27">
         <f t="shared" si="1"/>
-        <v>560</v>
-      </c>
-      <c r="E8" s="26">
-        <f>IF(C8="", "", H8-C8)</f>
-        <v>790</v>
-      </c>
-      <c r="F8" s="27">
-        <f>IF(H8="","",IF(C8="","",D8/(H8-C7)))</f>
         <v>0.4148148148148148</v>
       </c>
-      <c r="G8" s="63">
-        <f t="shared" si="0"/>
+      <c r="G8" s="60">
+        <f t="shared" si="2"/>
         <v>1350</v>
       </c>
       <c r="H8" s="35">
@@ -2495,19 +2507,19 @@
         <v>6407</v>
       </c>
       <c r="D9" s="26">
+        <f t="shared" si="3"/>
+        <v>797</v>
+      </c>
+      <c r="E9" s="26">
+        <f t="shared" si="0"/>
+        <v>593</v>
+      </c>
+      <c r="F9" s="27">
         <f t="shared" si="1"/>
-        <v>797</v>
-      </c>
-      <c r="E9" s="26">
-        <f>IF(C9="", "", H9-C9)</f>
-        <v>593</v>
-      </c>
-      <c r="F9" s="27">
-        <f>IF(H9="","",IF(C9="","",D9/(H9-C8)))</f>
         <v>0.57338129496402879</v>
       </c>
-      <c r="G9" s="63">
-        <f t="shared" si="0"/>
+      <c r="G9" s="60">
+        <f t="shared" si="2"/>
         <v>1390</v>
       </c>
       <c r="H9" s="35">
@@ -2525,19 +2537,19 @@
         <v>7066</v>
       </c>
       <c r="D10" s="28">
+        <f t="shared" si="3"/>
+        <v>659</v>
+      </c>
+      <c r="E10" s="28">
+        <f t="shared" si="0"/>
+        <v>934</v>
+      </c>
+      <c r="F10" s="33">
         <f t="shared" si="1"/>
-        <v>659</v>
-      </c>
-      <c r="E10" s="28">
-        <f>IF(C10="", "", H10-C10)</f>
-        <v>934</v>
-      </c>
-      <c r="F10" s="33">
-        <f>IF(H10="","",IF(C10="","",D10/(H10-C9)))</f>
         <v>0.41368487131198994</v>
       </c>
-      <c r="G10" s="66">
-        <f t="shared" si="0"/>
+      <c r="G10" s="63">
+        <f t="shared" si="2"/>
         <v>1593</v>
       </c>
       <c r="H10" s="36">
@@ -2551,23 +2563,23 @@
       <c r="B11" s="2">
         <v>46258</v>
       </c>
-      <c r="C11" s="67">
+      <c r="C11" s="64">
         <v>7218</v>
       </c>
       <c r="D11" s="26">
+        <f t="shared" si="3"/>
+        <v>152</v>
+      </c>
+      <c r="E11" s="26">
+        <f t="shared" si="0"/>
+        <v>1282</v>
+      </c>
+      <c r="F11" s="27">
         <f t="shared" si="1"/>
-        <v>152</v>
-      </c>
-      <c r="E11" s="26">
-        <f>IF(C11="", "", H11-C11)</f>
-        <v>1282</v>
-      </c>
-      <c r="F11" s="27">
-        <f>IF(H11="","",IF(C11="","",D11/(H11-C10)))</f>
         <v>0.10599721059972106</v>
       </c>
-      <c r="G11" s="63">
-        <f t="shared" si="0"/>
+      <c r="G11" s="60">
+        <f t="shared" si="2"/>
         <v>1434</v>
       </c>
       <c r="H11" s="35">
@@ -2585,19 +2597,19 @@
         <v>8459</v>
       </c>
       <c r="D12" s="28">
+        <f t="shared" si="3"/>
+        <v>1241</v>
+      </c>
+      <c r="E12" s="28">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="F12" s="33">
         <f t="shared" si="1"/>
-        <v>1241</v>
-      </c>
-      <c r="E12" s="28">
-        <f>IF(C12="", "", H12-C12)</f>
-        <v>41</v>
-      </c>
-      <c r="F12" s="33">
-        <f>IF(H12="","",IF(C12="","",D12/(H12-C11)))</f>
         <v>0.96801872074883</v>
       </c>
-      <c r="G12" s="66">
-        <f t="shared" si="0"/>
+      <c r="G12" s="63">
+        <f t="shared" si="2"/>
         <v>1282</v>
       </c>
       <c r="H12" s="36">
@@ -2615,19 +2627,19 @@
         <v>8780</v>
       </c>
       <c r="D13" s="26">
+        <f t="shared" si="3"/>
+        <v>321</v>
+      </c>
+      <c r="E13" s="26">
+        <f t="shared" si="0"/>
+        <v>1220</v>
+      </c>
+      <c r="F13" s="27">
         <f t="shared" si="1"/>
-        <v>321</v>
-      </c>
-      <c r="E13" s="26">
-        <f>IF(C13="", "", H13-C13)</f>
-        <v>1220</v>
-      </c>
-      <c r="F13" s="27">
-        <f>IF(H13="","",IF(C13="","",D13/(H13-C12)))</f>
         <v>0.20830629461388708</v>
       </c>
-      <c r="G13" s="63">
-        <f t="shared" si="0"/>
+      <c r="G13" s="60">
+        <f t="shared" si="2"/>
         <v>1541</v>
       </c>
       <c r="H13" s="35">
@@ -2642,7 +2654,6 @@
         <v>46261</v>
       </c>
       <c r="C14" s="40">
-        <f>Q$6</f>
         <v>9647</v>
       </c>
       <c r="D14" s="28">
@@ -2650,14 +2661,14 @@
         <v>867</v>
       </c>
       <c r="E14" s="28">
-        <f>IF(C14="", "", H14-C14)</f>
+        <f t="shared" si="0"/>
         <v>1353</v>
       </c>
       <c r="F14" s="33">
-        <f>IF(H14="","",IF(C14="","",D14/(H14-C13)))</f>
+        <f t="shared" si="1"/>
         <v>0.39054054054054055</v>
       </c>
-      <c r="G14" s="66">
+      <c r="G14" s="63">
         <f>H14-C13</f>
         <v>2220</v>
       </c>
@@ -2672,20 +2683,22 @@
       <c r="B15" s="2">
         <v>46262</v>
       </c>
-      <c r="C15" s="40"/>
-      <c r="D15" s="26" t="str">
+      <c r="C15" s="40">
+        <v>9647</v>
+      </c>
+      <c r="D15" s="26">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E15" s="26">
+        <f t="shared" si="0"/>
+        <v>-9647</v>
+      </c>
+      <c r="F15" s="27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E15" s="26" t="str">
-        <f>IF(C15="", "", H15-C15)</f>
-        <v/>
-      </c>
-      <c r="F15" s="27" t="str">
-        <f>IF(H15="","",IF(C15="","",D15/(H15-C14)))</f>
-        <v/>
-      </c>
-      <c r="G15" s="63"/>
+      <c r="G15" s="60"/>
       <c r="H15" s="35"/>
       <c r="I15" s="19">
         <v>20000</v>
@@ -2695,20 +2708,22 @@
       <c r="B16" s="2">
         <v>46263</v>
       </c>
-      <c r="C16" s="40"/>
-      <c r="D16" s="26" t="str">
+      <c r="C16" s="40">
+        <v>9647</v>
+      </c>
+      <c r="D16" s="26">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E16" s="26">
+        <f t="shared" si="0"/>
+        <v>-9647</v>
+      </c>
+      <c r="F16" s="27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E16" s="26" t="str">
-        <f>IF(C16="", "", H16-C16)</f>
-        <v/>
-      </c>
-      <c r="F16" s="27" t="str">
-        <f>IF(H16="","",IF(C16="","",D16/(H16-C15)))</f>
-        <v/>
-      </c>
-      <c r="G16" s="63"/>
+      <c r="G16" s="60"/>
       <c r="H16" s="35"/>
       <c r="I16" s="19">
         <v>20000</v>
@@ -2718,20 +2733,22 @@
       <c r="B17" s="4">
         <v>46264</v>
       </c>
-      <c r="C17" s="41"/>
-      <c r="D17" s="28" t="str">
+      <c r="C17" s="40">
+        <v>9647</v>
+      </c>
+      <c r="D17" s="28">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E17" s="28">
+        <f t="shared" si="0"/>
+        <v>-9647</v>
+      </c>
+      <c r="F17" s="33" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E17" s="28" t="str">
-        <f>IF(C17="", "", H17-C17)</f>
-        <v/>
-      </c>
-      <c r="F17" s="33" t="str">
-        <f>IF(H17="","",IF(C17="","",D17/(H17-C16)))</f>
-        <v/>
-      </c>
-      <c r="G17" s="66"/>
+      <c r="G17" s="63"/>
       <c r="H17" s="36"/>
       <c r="I17" s="20">
         <v>20000</v>
@@ -2741,21 +2758,26 @@
       <c r="B18" s="5">
         <v>46265</v>
       </c>
-      <c r="C18" s="42"/>
-      <c r="D18" s="29" t="str">
+      <c r="C18" s="42">
+        <f>Q6</f>
+        <v>11228</v>
+      </c>
+      <c r="D18" s="29">
+        <f t="shared" si="3"/>
+        <v>1581</v>
+      </c>
+      <c r="E18" s="29">
+        <f t="shared" si="0"/>
+        <v>772</v>
+      </c>
+      <c r="F18" s="30">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="E18" s="29" t="str">
-        <f>IF(C18="", "", H18-C18)</f>
-        <v/>
-      </c>
-      <c r="F18" s="30" t="str">
-        <f>IF(H18="","",IF(C18="","",D18/(H18-C17)))</f>
-        <v/>
-      </c>
-      <c r="G18" s="64"/>
-      <c r="H18" s="37"/>
+        <v>0.67190820229494264</v>
+      </c>
+      <c r="G18" s="61"/>
+      <c r="H18" s="37">
+        <v>12000</v>
+      </c>
       <c r="I18" s="21">
         <v>20000</v>
       </c>
@@ -2766,18 +2788,18 @@
       </c>
       <c r="C19" s="50"/>
       <c r="D19" s="51" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="E19" s="51" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F19" s="52" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E19" s="51" t="str">
-        <f>IF(C19="", "", H19-C19)</f>
-        <v/>
-      </c>
-      <c r="F19" s="52" t="str">
-        <f>IF(H19="","",IF(C19="","",D19/(H19-C18)))</f>
-        <v/>
-      </c>
-      <c r="G19" s="65"/>
+      <c r="G19" s="62"/>
       <c r="H19" s="50"/>
       <c r="I19" s="53">
         <v>20000</v>
@@ -2789,18 +2811,18 @@
       </c>
       <c r="C20" s="35"/>
       <c r="D20" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="E20" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F20" s="27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E20" s="26" t="str">
-        <f>IF(C20="", "", H20-C20)</f>
-        <v/>
-      </c>
-      <c r="F20" s="27" t="str">
-        <f>IF(H20="","",IF(C20="","",D20/(H20-C19)))</f>
-        <v/>
-      </c>
-      <c r="G20" s="63"/>
+      <c r="G20" s="60"/>
       <c r="H20" s="35"/>
       <c r="I20" s="19">
         <v>20000</v>
@@ -2812,18 +2834,18 @@
       </c>
       <c r="C21" s="41"/>
       <c r="D21" s="28" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="E21" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F21" s="33" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E21" s="28" t="str">
-        <f>IF(C21="", "", H21-C21)</f>
-        <v/>
-      </c>
-      <c r="F21" s="33" t="str">
-        <f>IF(H21="","",IF(C21="","",D21/(H21-C20)))</f>
-        <v/>
-      </c>
-      <c r="G21" s="66"/>
+      <c r="G21" s="63"/>
       <c r="H21" s="36"/>
       <c r="I21" s="20">
         <v>20000</v>
@@ -2835,18 +2857,18 @@
       </c>
       <c r="C22" s="40"/>
       <c r="D22" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="E22" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F22" s="27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E22" s="26" t="str">
-        <f>IF(C22="", "", H22-C22)</f>
-        <v/>
-      </c>
-      <c r="F22" s="27" t="str">
-        <f>IF(H22="","",IF(C22="","",D22/(H22-C21)))</f>
-        <v/>
-      </c>
-      <c r="G22" s="63"/>
+      <c r="G22" s="60"/>
       <c r="H22" s="35"/>
       <c r="I22" s="19">
         <v>20000</v>
@@ -2858,18 +2880,18 @@
       </c>
       <c r="C23" s="40"/>
       <c r="D23" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="E23" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F23" s="27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E23" s="26" t="str">
-        <f>IF(C23="", "", H23-C23)</f>
-        <v/>
-      </c>
-      <c r="F23" s="27" t="str">
-        <f>IF(H23="","",IF(C23="","",D23/(H23-C22)))</f>
-        <v/>
-      </c>
-      <c r="G23" s="63"/>
+      <c r="G23" s="60"/>
       <c r="H23" s="35"/>
       <c r="I23" s="19">
         <v>20000</v>
@@ -2881,18 +2903,18 @@
       </c>
       <c r="C24" s="41"/>
       <c r="D24" s="28" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="E24" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F24" s="33" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E24" s="28" t="str">
-        <f>IF(C24="", "", H24-C24)</f>
-        <v/>
-      </c>
-      <c r="F24" s="33" t="str">
-        <f>IF(H24="","",IF(C24="","",D24/(H24-C23)))</f>
-        <v/>
-      </c>
-      <c r="G24" s="66"/>
+      <c r="G24" s="63"/>
       <c r="H24" s="36"/>
       <c r="I24" s="20">
         <v>20000</v>
@@ -2904,18 +2926,18 @@
       </c>
       <c r="C25" s="40"/>
       <c r="D25" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="E25" s="26" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F25" s="27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E25" s="26" t="str">
-        <f>IF(C25="", "", H25-C25)</f>
-        <v/>
-      </c>
-      <c r="F25" s="27" t="str">
-        <f>IF(H25="","",IF(C25="","",D25/(H25-C24)))</f>
-        <v/>
-      </c>
-      <c r="G25" s="63"/>
+      <c r="G25" s="60"/>
       <c r="H25" s="35"/>
       <c r="I25" s="19">
         <v>20000</v>
@@ -2927,18 +2949,18 @@
       </c>
       <c r="C26" s="42"/>
       <c r="D26" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="E26" s="29" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F26" s="30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E26" s="29" t="str">
-        <f>IF(C26="", "", H26-C26)</f>
-        <v/>
-      </c>
-      <c r="F26" s="30" t="str">
-        <f>IF(H26="","",IF(C26="","",D26/(H26-C25)))</f>
-        <v/>
-      </c>
-      <c r="G26" s="64"/>
+      <c r="G26" s="61"/>
       <c r="H26" s="37"/>
       <c r="I26" s="21">
         <v>20000</v>
@@ -2950,18 +2972,18 @@
       </c>
       <c r="C27" s="38"/>
       <c r="D27" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="E27" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="F27" s="18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="E27" s="7" t="str">
-        <f>IF(C27="", "", H27-C27)</f>
-        <v/>
-      </c>
-      <c r="F27" s="18" t="str">
-        <f>IF(H27="","",IF(C27="","",D27/(H27-C26)))</f>
-        <v/>
-      </c>
-      <c r="G27" s="62"/>
+      <c r="G27" s="59"/>
       <c r="H27" s="38"/>
       <c r="I27" s="34">
         <v>20000</v>

</xml_diff>